<commit_message>
Conditional formatting: data bars (Tier 3, Fase B)
Adds eCondDataBar as a fourth rule type alongside cellIs/
duplicateValues/colorScale: each numeric cell fills a fraction of its
own width (not a blended color) proportional to where its value falls
between the range's min and max, reusing ColorScalePoint for the two
thresholds instead of a new struct. Wired end to end: a fourth type
in the Conditional Formatting dialog (one color, like Excel), live
evaluation and rendering in SheetView (drawn on top of any existing
background, text still legible), native persistence (ASCD version
bumped to 6), and XLSX import of <dataBar> reusing the same inline
cfvo/color parsing as <colorScale>. Icon sets are the next rule type
in this same effort, not included here.
</commit_message>
<xml_diff>
--- a/translators/xlsx/tests/sample_condformat.xlsx
+++ b/translators/xlsx/tests/sample_condformat.xlsx
@@ -117,5 +117,14 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="D1:D10">
+    <cfRule type="dataBar" priority="4">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FF638EC6"/>
+      </dataBar>
+    </cfRule>
+  </conditionalFormatting>
 </worksheet>
 </file>
</xml_diff>